<commit_message>
Update Revenue Opportunity regression cases
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Revenue_Opportunity_Regression.xlsx
+++ b/docs/Revenue_Opportunity_Regression.xlsx
@@ -1,12 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4BC6827-0D5A-455F-ACC9-E64E80DC7D68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Summary" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Regression TCs" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Notes" state="visible" r:id="rId6"/>
+    <sheet name="Summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Regression TCs" sheetId="2" r:id="rId2"/>
+    <sheet name="Notes" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -186,13 +190,13 @@
     <t>REG-RO-001 — Page loads via menu/route with correct breadcrumb</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Login to Blue Triangle portal
+    <t>1. Login to Blue Triangle portal
 2. Ensure site is "GDC Test Site 2" (US)
 3. Open left nav: Business Insights &gt; Improve Conversion &gt; Revenue Opportunity (or Favorites shortcut if present)
 4. Observe breadcrumb and URL</t>
   </si>
   <si>
-    <t xml:space="preserve">Breadcrumb shows Business Insights / Improve Conversion / Revenue Opportunity
+    <t>Breadcrumb shows Business Insights / Improve Conversion / Revenue Opportunity
 URL contains business-analytics/revenue-opportunity
 User remains authenticated</t>
   </si>
@@ -203,12 +207,12 @@
     <t>REG-RO-002 — Default report/session context renders opportunity widgets</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Open Revenue Opportunity
+    <t>1. Open Revenue Opportunity
 2. Note the default selected Report in the Report dropdown
 3. Observe 30 Day Opportunity cards and charts</t>
   </si>
   <si>
-    <t xml:space="preserve">A default report is selected
+    <t>A default report is selected
 Top opportunity / device cards are visible
 Highcharts containers render with data</t>
   </si>
@@ -219,11 +223,11 @@
     <t>REG-RO-003 — Page load performance: title + charts within SLA window</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Navigate to Revenue Opportunity from a warm session
+    <t>1. Navigate to Revenue Opportunity from a warm session
 2. Measure time until title and charts are ready</t>
   </si>
   <si>
-    <t xml:space="preserve">Page becomes interactive with charts within 120 seconds
+    <t>Page becomes interactive with charts within 120 seconds
 No blank shell / login redirect</t>
   </si>
   <si>
@@ -233,11 +237,11 @@
     <t>REG-RO-004 — Revenue Data Type: Web Browser Data refreshes widgets</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Set Revenue Data Type to Web Browser Data
+    <t>1. Set Revenue Data Type to Web Browser Data
 2. Wait for widgets/charts to refresh</t>
   </si>
   <si>
-    <t xml:space="preserve">Charts refresh successfully
+    <t>Charts refresh successfully
 Page title remains Revenue Opportunity</t>
   </si>
   <si>
@@ -247,11 +251,11 @@
     <t>REG-RO-005 — Revenue Data Type: Native App Data sample</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Set Revenue Data Type to Native App Data (if configured for site)
+    <t>1. Set Revenue Data Type to Native App Data (if configured for site)
 2. Observe refresh; if unavailable, fall back to Web Browser Data</t>
   </si>
   <si>
-    <t xml:space="preserve">Native App Data applies when configured OR fallback keeps page healthy
+    <t>Native App Data applies when configured OR fallback keeps page healthy
 Charts remain populated</t>
   </si>
   <si>
@@ -261,11 +265,11 @@
     <t>REG-RO-006 — Revenue Data Type: Web Browser &amp; Native App combination</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Select combined Web Browser &amp; Native App data type
+    <t>1. Select combined Web Browser &amp; Native App data type
 2. Confirm widgets refresh</t>
   </si>
   <si>
-    <t xml:space="preserve">Combined data type applies or safe fallback occurs
+    <t>Combined data type applies or safe fallback occurs
 Charts show data</t>
   </si>
   <si>
@@ -275,11 +279,11 @@
     <t>REG-RO-007 — Report Type sample combination refreshes page</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Change Report Type (e.g. Page Name)
+    <t>1. Change Report Type (e.g. Page Name)
 2. Change to another type if available (CWV Selector)</t>
   </si>
   <si>
-    <t xml:space="preserve">Report Type changes refresh page content
+    <t>Report Type changes refresh page content
 Charts remain healthy</t>
   </si>
   <si>
@@ -289,11 +293,11 @@
     <t>REG-RO-008 — Report dropdown: switch to second available report</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Open Report dropdown
+    <t>1. Open Report dropdown
 2. Select the second listed report (if more than one exists)</t>
   </si>
   <si>
-    <t xml:space="preserve">Selected report loads
+    <t>Selected report loads
 Opportunity widgets refresh</t>
   </si>
   <si>
@@ -303,11 +307,11 @@
     <t>REG-RO-009 — Restore primary/default report (index 0)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Select the first report in the Report list
+    <t>1. Select the first report in the Report list
 2. Confirm default-ish context returns</t>
   </si>
   <si>
-    <t xml:space="preserve">First report is active
+    <t>First report is active
 Default opportunity context is visible</t>
   </si>
   <si>
@@ -317,13 +321,13 @@
     <t>REG-RO-010 — All / Desktop / Mobile card clicks refresh sections</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click All / Browser opportunity card
+    <t>1. Click All / Browser opportunity card
 2. Click Desktop card
 3. Click Mobile card
 4. Observe graphs/tables refresh after each click</t>
   </si>
   <si>
-    <t xml:space="preserve">Each card click updates corresponding sections
+    <t>Each card click updates corresponding sections
 Charts remain populated after each selection</t>
   </si>
   <si>
@@ -333,12 +337,12 @@
     <t>REG-RO-011 — Revenue Opportunity By Page: graph visible + tooltip on hover</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Locate Revenue Opportunity By Page horizontal bar graph
+    <t>1. Locate Revenue Opportunity By Page horizontal bar graph
 2. Hover a bar/point
 3. Observe tooltip values</t>
   </si>
   <si>
-    <t xml:space="preserve">By Page graph is visible
+    <t>By Page graph is visible
 Tooltip shows revenue values on hover (when data allows)</t>
   </si>
   <si>
@@ -348,13 +352,13 @@
     <t>REG-RO-012 — Revenue Opportunity By Page: legend toggle + context menu</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Toggle a legend item under/near the By Page graph
+    <t>1. Toggle a legend item under/near the By Page graph
 2. Toggle it back
 3. Open chart hamburger/context menu
 4. Dismiss with Escape</t>
   </si>
   <si>
-    <t xml:space="preserve">Legend toggles series visibility
+    <t>Legend toggles series visibility
 Context menu chrome is available</t>
   </si>
   <si>
@@ -364,12 +368,12 @@
     <t>REG-RO-013 — Revenue Opportunity By Platform: hover tooltip + legend</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Locate By Platform bar graph
+    <t>1. Locate By Platform bar graph
 2. Hover for tooltip
 3. Toggle legend item check/uncheck</t>
   </si>
   <si>
-    <t xml:space="preserve">By Platform graph visible
+    <t>By Platform graph visible
 Tooltip/legend interactions refresh presentation</t>
   </si>
   <si>
@@ -379,7 +383,7 @@
     <t>REG-RO-014 — Revenue Opportunity By Platform: context menu</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Open hamburger/context menu on By Platform graph
+    <t>1. Open hamburger/context menu on By Platform graph
 2. Dismiss menu</t>
   </si>
   <si>
@@ -389,24 +393,24 @@
     <t>REG-RO-015 — Total Actual Revenue: hover tooltip + context menu</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Locate Total Actual Revenue bar graph
+    <t>1. Locate Total Actual Revenue bar graph
 2. Hover for exact values
 3. Open context menu and dismiss</t>
   </si>
   <si>
-    <t xml:space="preserve">Graph visible
+    <t>Graph visible
 Tooltip/menu interactions succeed or page stays healthy</t>
   </si>
   <si>
     <t>REG-RO-016 — All Browser Devices 30 days: line graph hover + legend</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Locate All Browser Devices / Actual Sales Over Time line graph
+    <t>1. Locate All Browser Devices / Actual Sales Over Time line graph
 2. Hover a point for day revenue
 3. Toggle legend; open context menu</t>
   </si>
   <si>
-    <t xml:space="preserve">Line graph visible
+    <t>Line graph visible
 Hover/legend/menu behaviors work as available</t>
   </si>
   <si>
@@ -416,11 +420,11 @@
     <t>REG-RO-017 — What If table visible with optimized/faster columns</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Scroll to What If table
+    <t>1. Scroll to What If table
 2. Confirm columns for optimized / Ns faster opportunity</t>
   </si>
   <si>
-    <t xml:space="preserve">What If / business overview table is visible
+    <t>What If / business overview table is visible
 Fully Optimized / What If faster columns are present</t>
   </si>
   <si>
@@ -430,12 +434,12 @@
     <t>REG-RO-018 — What If: edit variables then Cancel (no Save)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Hover What If variables and click pencil/edit
+    <t>1. Hover What If variables and click pencil/edit
 2. Change a sample second increment if editable
 3. Click Cancel (do NOT Save)</t>
   </si>
   <si>
-    <t xml:space="preserve">Edit UI opens
+    <t>Edit UI opens
 Cancel discards changes
 No persistent What If Save is performed (read-only automation rule)</t>
   </si>
@@ -446,11 +450,11 @@
     <t>REG-RO-019 — Column sort</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click a sortable column header (Page Name / Fully Optimized / Total Opportunity)
+    <t>1. Click a sortable column header (Page Name / Fully Optimized / Total Opportunity)
 2. Observe row order change</t>
   </si>
   <si>
-    <t xml:space="preserve">Column sort is applied
+    <t>Column sort is applied
 Table remains visible</t>
   </si>
   <si>
@@ -460,11 +464,11 @@
     <t>REG-RO-020 — Search/filter</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Use table search or column filter input
+    <t>1. Use table search or column filter input
 2. Enter a sample term</t>
   </si>
   <si>
-    <t xml:space="preserve">Search/filter narrows rows when control exists
+    <t>Search/filter narrows rows when control exists
 Table remains healthy</t>
   </si>
   <si>
@@ -474,11 +478,11 @@
     <t>REG-RO-021 — Pager navigation when present</t>
   </si>
   <si>
-    <t xml:space="preserve">1. If pager controls exist, click next
+    <t>1. If pager controls exist, click next
 2. Confirm table still visible</t>
   </si>
   <si>
-    <t xml:space="preserve">Pager advances when available
+    <t>Pager advances when available
 Table remains visible</t>
   </si>
   <si>
@@ -488,11 +492,11 @@
     <t>REG-RO-022 — Information icon tooltips sample</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Locate info icons near labels/fields
+    <t>1. Locate info icons near labels/fields
 2. Hover several icons and read tooltips</t>
   </si>
   <si>
-    <t xml:space="preserve">At least one info icon is hoverable
+    <t>At least one info icon is hoverable
 Tooltip/title text is exposed</t>
   </si>
   <si>
@@ -502,12 +506,12 @@
     <t>REG-RO-023 — View Filters / Hide Filters toggles applied-filter banner</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click View Filters
+    <t>1. Click View Filters
 2. Observe applied filter banner
 3. Click Hide Filters</t>
   </si>
   <si>
-    <t xml:space="preserve">Banner shows/hides
+    <t>Banner shows/hides
 Button label toggles View/Hide Filters</t>
   </si>
   <si>
@@ -517,25 +521,25 @@
     <t>REG-RO-024 — Right-nav Filters: performance metric + visitor type sample</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Open Filters (funnel) top-right
+    <t>1. Open Filters (funnel) top-right
 2. Set Performance Metric = Onload; Visitor Type = New Visitors; Apply
 3. Set Returning Visitors; Apply
 4. Do NOT Save Filter</t>
   </si>
   <si>
-    <t xml:space="preserve">Charts refresh for sampled filter combos
+    <t>Charts refresh for sampled filter combos
 No Save Filter write</t>
   </si>
   <si>
     <t>REG-RO-025 — Report Manager opens (read-only; no delete)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click Report Manager
+    <t>1. Click Report Manager
 2. Observe panel
 3. Close without deleting reports</t>
   </si>
   <si>
-    <t xml:space="preserve">Report Manager opens
+    <t>Report Manager opens
 No delete/write actions performed</t>
   </si>
   <si>
@@ -545,22 +549,22 @@
     <t>REG-RO-026 — Top-nav right controls visible with tooltips</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Hover Filters / Help Center / User menu (and other right-nav icons)
+    <t>1. Hover Filters / Help Center / User menu (and other right-nav icons)
 2. Confirm tooltips</t>
   </si>
   <si>
-    <t xml:space="preserve">Right-nav controls visible with tooltips
+    <t>Right-nav controls visible with tooltips
 Filters control remains available</t>
   </si>
   <si>
     <t>REG-RO-027 — Common legend check/uncheck refreshes series</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click a Highcharts legend item
+    <t>1. Click a Highcharts legend item
 2. Click again to restore</t>
   </si>
   <si>
-    <t xml:space="preserve">Series visibility toggles
+    <t>Series visibility toggles
 Charts remain populated</t>
   </si>
   <si>
@@ -570,18 +574,18 @@
     <t>REG-RO-028 — Additional UI: opportunity calculator / conversion graphs present</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Locate conversion / opportunity calculator graphs if rendered
+    <t>1. Locate conversion / opportunity calculator graphs if rendered
 2. Confirm visibility</t>
   </si>
   <si>
-    <t xml:space="preserve">Available calculator/conversion graphs are visible
+    <t>Available calculator/conversion graphs are visible
 Main charts still have data</t>
   </si>
   <si>
     <t>REG-RO-029 — Data refresh after device card + data type combo</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Set Revenue Data Type to Web Browser Data
+    <t>1. Set Revenue Data Type to Web Browser Data
 2. Click Desktop then All opportunity cards</t>
   </si>
   <si>
@@ -594,11 +598,11 @@
     <t>REG-RO-030 — Performance re-check after interactions: charts still load</t>
   </si>
   <si>
-    <t xml:space="preserve">1. After prior interactions, poll for chart containers
+    <t>1. After prior interactions, poll for chart containers
 2. Confirm title still Revenue Opportunity</t>
   </si>
   <si>
-    <t xml:space="preserve">Charts remain available within 60s poll
+    <t>Charts remain available within 60s poll
 Page title unchanged</t>
   </si>
   <si>
@@ -608,12 +612,12 @@
     <t>REG-RO-031 — iOS / Android card sample when present</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click iOS opportunity card (if present)
+    <t>1. Click iOS opportunity card (if present)
 2. Click Android opportunity card (if present)
 3. Return to All card</t>
   </si>
   <si>
-    <t xml:space="preserve">Device cards refresh charts when available
+    <t>Device cards refresh charts when available
 All card restores overview</t>
   </si>
   <si>
@@ -623,7 +627,7 @@
     <t>REG-RO-032 — Device overview table follows Desktop card selection</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click Desktop 30 Day Opportunity card
+    <t>1. Click Desktop 30 Day Opportunity card
 2. Confirm desktop business overview table is present</t>
   </si>
   <si>
@@ -636,11 +640,11 @@
     <t>REG-RO-033 — What If Save control present but unused (read-only guard)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Locate Save What If control if rendered
+    <t>1. Locate Save What If control if rendered
 2. Do NOT click Save</t>
   </si>
   <si>
-    <t xml:space="preserve">Save control may be present
+    <t>Save control may be present
 Automation does not persist What If changes</t>
   </si>
   <si>
@@ -650,7 +654,7 @@
     <t>REG-RO-034 — View Filters banner shows applied filter chip sample</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click View Filters
+    <t>1. Click View Filters
 2. Read applied filter chips (Real User / Time Period / Device / etc.)
 3. Hide Filters</t>
   </si>
@@ -664,7 +668,7 @@
     <t>REG-RO-035 — Revenue Calibration top-nav control is present (tooltip)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Locate Revenue Calibration control in top-right chrome
+    <t>1. Locate Revenue Calibration control in top-right chrome
 2. Hover and confirm tooltip</t>
   </si>
   <si>
@@ -677,14 +681,14 @@
     <t>REG-RO-036 — Time Period 1 Days: labels + Actual Revenue timeline</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Open Revenue Opportunity (no Bucket Size control on this page)
+    <t>1. Open Revenue Opportunity (no Bucket Size control on this page)
 2. Apply Time Period = 1 Day via matching Report (e.g. "… 1 Day …") or Filters Time Period if available
 3. Confirm Opportunity / Actual Revenue Over Time / What If labels mention 1 Day
 4. Hover Actual Revenue Over Time left→right
 5. Validate Highcharts x-axis day buckets (~1 day steps)</t>
   </si>
   <si>
-    <t xml:space="preserve">Period applied via Report list and/or Filters Time Period only (no Bucket Size)
+    <t>Period applied via Report list and/or Filters Time Period only (no Bucket Size)
 Labels show 1 Day Opportunity / Actual Revenue Over Time period text
 What If / opportunity widgets mention 1 day when present
 Actual Revenue timeline uses ~1-day buckets ending near now
@@ -697,12 +701,12 @@
     <t>REG-RO-037 — Time Period 7 Days: labels + Actual Revenue timeline</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Apply Time Period = 7 Days via Report matching "7 Days" (or Filters)
+    <t>1. Apply Time Period = 7 Days via Report matching "7 Days" (or Filters)
 2. Confirm Opportunity / Actual Revenue / What If period labels
 3. Hover Actual Revenue; validate ~1-day timeline buckets</t>
   </si>
   <si>
-    <t xml:space="preserve">No Bucket Size selection (control not present on Revenue Opportunity)
+    <t>No Bucket Size selection (control not present on Revenue Opportunity)
 Labels and widgets reflect 7 Days
 Actual Revenue timeline remains healthy with day-scale buckets</t>
   </si>
@@ -713,12 +717,12 @@
     <t>REG-RO-038 — Time Period 14 Days: labels + Actual Revenue timeline</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Apply Time Period = 14 Days via Report / Filters
+    <t>1. Apply Time Period = 14 Days via Report / Filters
 2. Confirm period labels on Opportunity, Actual Revenue Over Time, What If
 3. Validate Actual Revenue timeline buckets</t>
   </si>
   <si>
-    <t xml:space="preserve">Period applied without Bucket Size
+    <t>Period applied without Bucket Size
 UI labels mention 14 Days
 Timeline buckets remain ~1 day for multi-day reports</t>
   </si>
@@ -729,13 +733,13 @@
     <t>REG-RO-039 — Time Period 30 days: labels + Actual Revenue timeline</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Apply Time Period = 30 Days via Report matching "30 Days" (common default report)
+    <t>1. Apply Time Period = 30 Days via Report matching "30 Days" (common default report)
 2. Confirm "30 Day Opportunity" and Actual Revenue Over Time period text
 3. Confirm What If widgets mention 30 days when labeled
 4. Hover Actual Revenue; validate day buckets near now</t>
   </si>
   <si>
-    <t xml:space="preserve">30-day report/period applies; no Bucket Size control used
+    <t>30-day report/period applies; no Bucket Size control used
 Opportunity / Actual Revenue / What If labels align with 30 days
 Actual Revenue Over Time uses ~1-day Highcharts buckets ending near local now</t>
   </si>
@@ -761,28 +765,33 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -804,6 +813,12 @@
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -817,9 +832,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -829,6 +843,11 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1167,9 +1186,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E24"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -1177,327 +1196,327 @@
     <col min="4" max="4" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2"/>
-      <c r="C2"/>
-      <c r="D2"/>
-    </row>
-    <row r="3" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+    </row>
+    <row r="3" spans="1:5" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
+    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="4" t="s">
+    <row r="5" spans="1:5" s="3" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="B5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>4</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="4" t="s">
+    <row r="6" spans="1:5" s="3" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>4</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="4" t="s">
+    <row r="7" spans="1:5" s="3" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>3</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="4" t="s">
+    <row r="8" spans="1:5" s="3" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="B8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>3</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="4" t="s">
+    <row r="9" spans="1:5" s="3" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="3">
         <v>3</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="4" t="s">
+    <row r="10" spans="1:5" s="3" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>3</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="4" t="s">
+    <row r="11" spans="1:5" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="B11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <v>2</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="4" t="s">
+    <row r="12" spans="1:5" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="3">
         <v>2</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="4" t="s">
+    <row r="13" spans="1:5" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="3">
         <v>2</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14" s="4" t="s">
+    <row r="14" spans="1:5" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="3">
         <v>2</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="4" t="s">
+    <row r="15" spans="1:5" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="3">
         <v>2</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="4" t="s">
+    <row r="16" spans="1:5" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="3">
         <v>2</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" s="4" t="s">
+    <row r="17" spans="2:5" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="3">
         <v>1</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" s="4" t="s">
+    <row r="18" spans="2:5" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="3">
         <v>1</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="4" t="s">
+    <row r="19" spans="2:5" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="3">
         <v>1</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="4" t="s">
+    <row r="20" spans="2:5" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="3">
         <v>1</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" s="4" t="s">
+    <row r="21" spans="2:5" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B21" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="3">
         <v>1</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="4" t="s">
+    <row r="22" spans="2:5" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B22" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="3">
         <v>1</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="4" t="s">
+    <row r="23" spans="2:5" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B23" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="3">
         <v>1</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="3" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="5" t="s">
+    <row r="24" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="4">
         <v>39</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="4" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1507,14 +1526,14 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H40"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1525,1070 +1544,1067 @@
     <col min="8" max="8" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="B2" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="H2" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="H2" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="B3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="H3" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="B4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="H4" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="B5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="H5" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="B6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="7" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="H6" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="B7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="8" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="H7" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="B8" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="H8" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="H8" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="B9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="H9" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="B10" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="H10" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="H10" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="B11" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="H11" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="12" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="H11" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="B12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="H12" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="13" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="H12" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="4" t="s">
+      <c r="B13" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="H13" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="14" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="H13" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="B14" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="H14" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="H14" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15" s="4" t="s">
+      <c r="B15" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="H15" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="16" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="H15" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" s="4" t="s">
+      <c r="B16" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="H16" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="H16" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="4" t="s">
+      <c r="B17" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="H17" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="18" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="H17" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="B18" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="H18" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="H18" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19" s="4" t="s">
+      <c r="B19" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="H19" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="20" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="H19" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D20" s="4" t="s">
+      <c r="B20" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="H20" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="H20" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="B21" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="H21" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="22" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="H21" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="B22" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="H22" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="23" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="H22" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="4" t="s">
+      <c r="B23" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="H23" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+      <c r="H23" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="B24" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="H24" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="25" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="H24" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="4" t="s">
+      <c r="B25" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="H25" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="26" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+      <c r="H25" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="B26" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="H26" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+      <c r="H26" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" s="4" t="s">
+      <c r="B27" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="H27" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="28" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+      <c r="H27" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D28" s="4" t="s">
+      <c r="B28" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="H28" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="29" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+      <c r="H28" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D29" s="4" t="s">
+      <c r="B29" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="F29" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="G29" s="4" t="s">
+      <c r="G29" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="H29" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
+      <c r="H29" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" s="4" t="s">
+      <c r="B30" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="G30" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="H30" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="31" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+      <c r="H30" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="B31" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D31" s="4" t="s">
+      <c r="B31" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="F31" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="G31" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="H31" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="32" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+      <c r="H31" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="B32" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32" s="4" t="s">
+      <c r="B32" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E32" s="4" t="s">
+      <c r="E32" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="F32" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="G32" s="4" t="s">
+      <c r="G32" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="H32" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="33" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
+      <c r="H32" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="B33" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D33" s="4" t="s">
+      <c r="B33" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E33" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F33" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="G33" s="4" t="s">
+      <c r="G33" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="H33" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="34" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
+      <c r="H33" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="B34" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D34" s="4" t="s">
+      <c r="B34" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D34" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F34" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="G34" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="H34" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="35" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
+      <c r="H34" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D35" s="4" t="s">
+      <c r="B35" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="E35" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="F35" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="G35" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="H35" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="36" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
+      <c r="H35" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="B36" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D36" s="4" t="s">
+      <c r="B36" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E36" s="4" t="s">
+      <c r="E36" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="F36" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="G36" s="4" t="s">
+      <c r="G36" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="H36" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="37" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
+      <c r="H36" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="B37" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D37" s="4" t="s">
+      <c r="B37" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="E37" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F37" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="G37" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="H37" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="38" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
+      <c r="H37" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D38" s="4" t="s">
+      <c r="B38" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E38" s="4" t="s">
+      <c r="E38" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="F38" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="G38" s="4" t="s">
+      <c r="G38" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="H38" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="39" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
+      <c r="H38" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D39" s="4" t="s">
+      <c r="B39" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E39" s="4" t="s">
+      <c r="E39" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="F39" s="4" t="s">
+      <c r="F39" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="G39" s="4" t="s">
+      <c r="G39" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="H39" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="40" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
+      <c r="H39" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="3" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D40" s="4" t="s">
+      <c r="B40" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E40" s="4" t="s">
+      <c r="E40" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="F40" s="4" t="s">
+      <c r="F40" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="G40" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="H40" s="4" t="s">
+      <c r="H40" s="3" t="s">
         <v>59</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="H10:H40">
-      <formula1>"Not Executed,Pass,Fail,Blocked,Skipped"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2:H40">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Not Executed,Pass,Fail,Blocked,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>206</v>
       </c>
     </row>
@@ -2624,6 +2640,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>